<commit_message>
Fix item counts for ID 49 subscales
</commit_message>
<xml_diff>
--- a/Full text coding sheet.xlsx
+++ b/Full text coding sheet.xlsx
@@ -582,7 +582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX1192"/>
+  <dimension ref="A1:AX1193"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.22" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.67" customWidth="1" style="35" min="1" max="4"/>
@@ -18318,7 +18318,7 @@
       <c r="AK1171" s="11" t="n"/>
     </row>
     <row r="1172">
-      <c r="B1172" t="n">
+      <c r="B1172" s="0" t="n">
         <v>49</v>
       </c>
       <c r="C1172" s="0" t="n">
@@ -18333,7 +18333,7 @@
         </is>
       </c>
       <c r="AA1172" s="0" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="AB1172" s="0" t="n">
         <v>999</v>
@@ -18408,7 +18408,7 @@
       </c>
     </row>
     <row r="1173">
-      <c r="B1173" t="n">
+      <c r="B1173" s="0" t="n">
         <v>49</v>
       </c>
       <c r="C1173" s="0" t="n">
@@ -18423,7 +18423,7 @@
         </is>
       </c>
       <c r="AA1173" s="0" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="AB1173" s="0" t="n">
         <v>999</v>
@@ -18498,7 +18498,7 @@
       </c>
     </row>
     <row r="1174">
-      <c r="B1174" t="n">
+      <c r="B1174" s="0" t="n">
         <v>49</v>
       </c>
       <c r="C1174" s="0" t="n">
@@ -18513,7 +18513,7 @@
         </is>
       </c>
       <c r="AA1174" s="0" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="AB1174" s="0" t="n">
         <v>999</v>
@@ -18588,7 +18588,7 @@
       </c>
     </row>
     <row r="1175">
-      <c r="B1175" t="n">
+      <c r="B1175" s="0" t="n">
         <v>49</v>
       </c>
       <c r="C1175" s="0" t="n">
@@ -18603,7 +18603,7 @@
         </is>
       </c>
       <c r="AA1175" s="0" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="AB1175" s="0" t="n">
         <v>999</v>
@@ -18678,7 +18678,7 @@
       </c>
     </row>
     <row r="1176">
-      <c r="B1176" t="n">
+      <c r="B1176" s="0" t="n">
         <v>49</v>
       </c>
       <c r="C1176" s="0" t="n">
@@ -18693,7 +18693,7 @@
         </is>
       </c>
       <c r="AA1176" s="0" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="AB1176" s="0" t="n">
         <v>999</v>
@@ -18768,7 +18768,7 @@
       </c>
     </row>
     <row r="1177">
-      <c r="B1177" t="n">
+      <c r="B1177" s="0" t="n">
         <v>49</v>
       </c>
       <c r="C1177" s="0" t="n">
@@ -18783,7 +18783,7 @@
         </is>
       </c>
       <c r="AA1177" s="0" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="AB1177" s="0" t="n">
         <v>999</v>
@@ -18858,7 +18858,7 @@
       </c>
     </row>
     <row r="1178">
-      <c r="B1178" t="n">
+      <c r="B1178" s="0" t="n">
         <v>49</v>
       </c>
       <c r="C1178" s="0" t="n">
@@ -18873,7 +18873,7 @@
         </is>
       </c>
       <c r="AA1178" s="0" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="AB1178" s="0" t="n">
         <v>999</v>
@@ -18948,7 +18948,7 @@
       </c>
     </row>
     <row r="1179">
-      <c r="B1179" t="n">
+      <c r="B1179" s="0" t="n">
         <v>49</v>
       </c>
       <c r="C1179" s="0" t="n">
@@ -18963,7 +18963,7 @@
         </is>
       </c>
       <c r="AA1179" s="0" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="AB1179" s="0" t="n">
         <v>999</v>
@@ -19038,7 +19038,7 @@
       </c>
     </row>
     <row r="1180">
-      <c r="B1180" t="n">
+      <c r="B1180" s="0" t="n">
         <v>49</v>
       </c>
       <c r="C1180" s="0" t="n">
@@ -19053,7 +19053,7 @@
         </is>
       </c>
       <c r="AA1180" s="0" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="AB1180" s="0" t="n">
         <v>999</v>
@@ -19128,7 +19128,7 @@
       </c>
     </row>
     <row r="1181">
-      <c r="B1181" t="n">
+      <c r="B1181" s="0" t="n">
         <v>49</v>
       </c>
       <c r="C1181" s="0" t="n">
@@ -19143,7 +19143,7 @@
         </is>
       </c>
       <c r="AA1181" s="0" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="AB1181" s="0" t="n">
         <v>999</v>
@@ -19218,7 +19218,7 @@
       </c>
     </row>
     <row r="1182">
-      <c r="B1182" t="n">
+      <c r="B1182" s="0" t="n">
         <v>49</v>
       </c>
       <c r="C1182" s="0" t="n">
@@ -19233,7 +19233,7 @@
         </is>
       </c>
       <c r="AA1182" s="0" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AB1182" s="0" t="n">
         <v>999</v>
@@ -19308,7 +19308,7 @@
       </c>
     </row>
     <row r="1183">
-      <c r="B1183" t="n">
+      <c r="B1183" s="0" t="n">
         <v>49</v>
       </c>
       <c r="C1183" s="0" t="n">
@@ -19323,7 +19323,7 @@
         </is>
       </c>
       <c r="AA1183" s="0" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AB1183" s="0" t="n">
         <v>999</v>
@@ -19398,7 +19398,7 @@
       </c>
     </row>
     <row r="1184">
-      <c r="B1184" t="n">
+      <c r="B1184" s="0" t="n">
         <v>49</v>
       </c>
       <c r="C1184" s="0" t="n">
@@ -19413,7 +19413,7 @@
         </is>
       </c>
       <c r="AA1184" s="0" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AB1184" s="0" t="n">
         <v>999</v>
@@ -19488,7 +19488,7 @@
       </c>
     </row>
     <row r="1185">
-      <c r="B1185" t="n">
+      <c r="B1185" s="0" t="n">
         <v>49</v>
       </c>
       <c r="C1185" s="0" t="n">
@@ -19503,7 +19503,7 @@
         </is>
       </c>
       <c r="AA1185" s="0" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AB1185" s="0" t="n">
         <v>999</v>
@@ -19578,7 +19578,7 @@
       </c>
     </row>
     <row r="1186">
-      <c r="B1186" t="n">
+      <c r="B1186" s="0" t="n">
         <v>49</v>
       </c>
       <c r="C1186" s="0" t="n">
@@ -19593,7 +19593,7 @@
         </is>
       </c>
       <c r="AA1186" s="0" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AB1186" s="0" t="n">
         <v>999</v>
@@ -19668,7 +19668,7 @@
       </c>
     </row>
     <row r="1187">
-      <c r="B1187" t="n">
+      <c r="B1187" s="0" t="n">
         <v>53</v>
       </c>
       <c r="C1187" s="0" t="n">
@@ -19754,7 +19754,7 @@
       <c r="AX1187" s="0" t="inlineStr"/>
     </row>
     <row r="1188">
-      <c r="B1188" t="n">
+      <c r="B1188" s="0" t="n">
         <v>53</v>
       </c>
       <c r="C1188" s="0" t="n">
@@ -19840,7 +19840,7 @@
       <c r="AX1188" s="0" t="inlineStr"/>
     </row>
     <row r="1189">
-      <c r="B1189" t="n">
+      <c r="B1189" s="0" t="n">
         <v>53</v>
       </c>
       <c r="C1189" s="0" t="n">
@@ -19926,7 +19926,7 @@
       <c r="AX1189" s="0" t="inlineStr"/>
     </row>
     <row r="1190">
-      <c r="B1190" t="n">
+      <c r="B1190" s="0" t="n">
         <v>53</v>
       </c>
       <c r="C1190" s="0" t="n">
@@ -20012,7 +20012,7 @@
       <c r="AX1190" s="0" t="inlineStr"/>
     </row>
     <row r="1191">
-      <c r="B1191" t="n">
+      <c r="B1191" s="0" t="n">
         <v>53</v>
       </c>
       <c r="C1191" s="0" t="n">
@@ -20098,7 +20098,7 @@
       <c r="AX1191" s="0" t="inlineStr"/>
     </row>
     <row r="1192">
-      <c r="B1192" t="n">
+      <c r="B1192" s="0" t="n">
         <v>53</v>
       </c>
       <c r="C1192" s="0" t="n">
@@ -20182,6 +20182,29 @@
         <v>0.02</v>
       </c>
       <c r="AX1192" s="0" t="inlineStr"/>
+    </row>
+    <row r="1193">
+      <c r="B1193" s="0" t="n">
+        <v>66</v>
+      </c>
+      <c r="C1193" s="0" t="n">
+        <v>66</v>
+      </c>
+      <c r="E1193" s="0" t="inlineStr">
+        <is>
+          <t>0 = exclude</t>
+        </is>
+      </c>
+      <c r="F1193" s="0" t="inlineStr">
+        <is>
+          <t>Level of Analysis</t>
+        </is>
+      </c>
+      <c r="P1193" s="0" t="inlineStr">
+        <is>
+          <t>[Level of Analysis violation]. Verbatim Evidence: "[Methodology] Project leaders were required to complete the questionnaire with reference to a completed NPD project." "[Abstract] A Partial Least Squares test on 73 NPD projects showed that..."</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="$A$3:$AX$253"/>

</xml_diff>